<commit_message>
DFT program did not for MATRIX 1
DFT program did not do a MATRIX 1 at the end of Prog B and will cause user an get an Error 3 if they try to RCL Matrix A or B right after running.  Setting MATRIX 1 will avoid confusion to user and save time.  Also, delete the .hex files since we moved on to using the PH15C_Unterface.xls tool.
</commit_message>
<xml_diff>
--- a/engineering_basics/dft/forward_dft.xlsx
+++ b/engineering_basics/dft/forward_dft.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="196">
   <si>
     <t xml:space="preserve">Line Num</t>
   </si>
@@ -2255,11 +2255,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="62616022"/>
-        <c:axId val="47407687"/>
+        <c:axId val="33574547"/>
+        <c:axId val="53458440"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="62616022"/>
+        <c:axId val="33574547"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2336,12 +2336,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47407687"/>
+        <c:crossAx val="53458440"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="47407687"/>
+        <c:axId val="53458440"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2418,7 +2418,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62616022"/>
+        <c:crossAx val="33574547"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2481,9 +2481,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>546840</xdr:colOff>
+      <xdr:colOff>546480</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>28080</xdr:rowOff>
+      <xdr:rowOff>27720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2492,7 +2492,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="3963600" y="380160"/>
-        <a:ext cx="9778680" cy="5500080"/>
+        <a:ext cx="9778320" cy="5499720"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2616,7 +2616,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="14.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
@@ -4560,13 +4560,13 @@
     </row>
     <row r="76" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="11" t="n">
-        <v>74</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C76" s="21" t="s">
-        <v>130</v>
+        <v>75</v>
+      </c>
+      <c r="B76" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>174</v>
@@ -4581,17 +4581,43 @@
         <v>35</v>
       </c>
       <c r="H76" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C77" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H77" s="4" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="23"/>
-      <c r="B77" s="24"/>
-      <c r="C77" s="25"/>
-      <c r="D77" s="24"/>
-      <c r="E77" s="24"/>
-      <c r="F77" s="24"/>
-      <c r="G77" s="24"/>
+    <row r="78" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="23"/>
+      <c r="B78" s="24"/>
+      <c r="C78" s="25"/>
+      <c r="D78" s="24"/>
+      <c r="E78" s="24"/>
+      <c r="F78" s="24"/>
+      <c r="G78" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4600,7 +4626,7 @@
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="C1:C2 C4:C723">
+  <conditionalFormatting sqref="C1:C2 C4:C724">
     <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="uSTO C" dxfId="0">
       <formula>NOT(ISERROR(SEARCH("uSTO C",C1)))</formula>
     </cfRule>
@@ -4611,7 +4637,7 @@
       <formula>NOT(ISERROR(SEARCH("uSTO B",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C2 C4:C732">
+  <conditionalFormatting sqref="C1:C2 C4:C733">
     <cfRule type="containsText" priority="5" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="uSTO A" dxfId="0">
       <formula>NOT(ISERROR(SEARCH("uSTO A",C1)))</formula>
     </cfRule>

</xml_diff>